<commit_message>
Updated the excel data
</commit_message>
<xml_diff>
--- a/data/inventory.xlsx
+++ b/data/inventory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naveenkumar.P\Downloads\local_store_assistant_mvp_code\local_store_assistant_mvp\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://musigma-my.sharepoint.com/personal/devprasath_c_mu-sigma_com/Documents/Desktop/NV_ChatBot/Whatsapp_ChatBot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2112E095-9499-45D3-BFCC-076556098D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{2112E095-9499-45D3-BFCC-076556098D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07C525C0-3D02-4694-94C7-3A2201BE69B5}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A094C0FE-B072-46D8-B51B-241A0B2B1CC1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A094C0FE-B072-46D8-B51B-241A0B2B1CC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory_Data" sheetId="2" r:id="rId1"/>
@@ -1922,18 +1922,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2F73202-0479-4D18-A531-70D1AC27E9E6}">
   <dimension ref="A1:G139"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.26953125" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.90625" customWidth="1"/>
-    <col min="7" max="7" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1956,7 +1956,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1973,13 +1973,13 @@
         <v>32</v>
       </c>
       <c r="F2" s="2">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -2117,7 +2117,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -2163,7 +2163,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>35</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>42</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>42</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>50</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>50</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>50</v>
       </c>
@@ -2370,7 +2370,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>58</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>58</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>58</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>67</v>
       </c>
@@ -2462,7 +2462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>67</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>67</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>76</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>76</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>76</v>
       </c>
@@ -2577,7 +2577,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>85</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>85</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>85</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>93</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>93</v>
       </c>
@@ -2692,7 +2692,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>93</v>
       </c>
@@ -2715,7 +2715,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>103</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>103</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>103</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>112</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>112</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>112</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>121</v>
       </c>
@@ -2876,7 +2876,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>121</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>121</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>126</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>126</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>126</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>133</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>133</v>
       </c>
@@ -3037,7 +3037,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>133</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>139</v>
       </c>
@@ -3083,7 +3083,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>139</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>139</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>146</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>146</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>146</v>
       </c>
@@ -3198,7 +3198,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>153</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>153</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>153</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>159</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>159</v>
       </c>
@@ -3313,7 +3313,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>159</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>166</v>
       </c>
@@ -3359,7 +3359,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>166</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>166</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>173</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>173</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>173</v>
       </c>
@@ -3474,7 +3474,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>177</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>177</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>177</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>186</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>186</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>186</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>190</v>
       </c>
@@ -3635,7 +3635,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>190</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>190</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>195</v>
       </c>
@@ -3704,7 +3704,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>195</v>
       </c>
@@ -3727,7 +3727,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>195</v>
       </c>
@@ -3750,7 +3750,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>201</v>
       </c>
@@ -3773,7 +3773,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>201</v>
       </c>
@@ -3796,7 +3796,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>201</v>
       </c>
@@ -3819,7 +3819,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>207</v>
       </c>
@@ -3842,7 +3842,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>207</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>207</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>214</v>
       </c>
@@ -3911,7 +3911,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>214</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>214</v>
       </c>
@@ -3957,7 +3957,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>222</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>222</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>222</v>
       </c>
@@ -4026,7 +4026,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>229</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>229</v>
       </c>
@@ -4072,7 +4072,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>229</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>236</v>
       </c>
@@ -4118,7 +4118,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>236</v>
       </c>
@@ -4141,7 +4141,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>236</v>
       </c>
@@ -4164,7 +4164,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>245</v>
       </c>
@@ -4187,7 +4187,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>245</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>245</v>
       </c>
@@ -4233,7 +4233,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>252</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>252</v>
       </c>
@@ -4279,7 +4279,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>252</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>260</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>260</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>260</v>
       </c>
@@ -4371,7 +4371,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>265</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>265</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>265</v>
       </c>
@@ -4440,7 +4440,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>270</v>
       </c>
@@ -4463,7 +4463,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>270</v>
       </c>
@@ -4486,7 +4486,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>270</v>
       </c>
@@ -4509,7 +4509,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>276</v>
       </c>
@@ -4532,7 +4532,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>276</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>276</v>
       </c>
@@ -4578,7 +4578,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>284</v>
       </c>
@@ -4601,7 +4601,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>284</v>
       </c>
@@ -4624,7 +4624,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>284</v>
       </c>
@@ -4647,7 +4647,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>290</v>
       </c>
@@ -4670,7 +4670,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>290</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>290</v>
       </c>
@@ -4716,7 +4716,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>297</v>
       </c>
@@ -4739,7 +4739,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>297</v>
       </c>
@@ -4762,7 +4762,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>297</v>
       </c>
@@ -4785,7 +4785,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>303</v>
       </c>
@@ -4808,7 +4808,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>303</v>
       </c>
@@ -4831,7 +4831,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>303</v>
       </c>
@@ -4854,7 +4854,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>312</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>312</v>
       </c>
@@ -4900,7 +4900,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>312</v>
       </c>
@@ -4923,7 +4923,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>318</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>318</v>
       </c>
@@ -4969,7 +4969,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>318</v>
       </c>
@@ -4992,7 +4992,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>324</v>
       </c>
@@ -5015,7 +5015,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>324</v>
       </c>
@@ -5038,7 +5038,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>324</v>
       </c>
@@ -5061,7 +5061,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>332</v>
       </c>
@@ -5084,7 +5084,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>332</v>
       </c>
@@ -5107,7 +5107,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>332</v>
       </c>

</xml_diff>